<commit_message>
EBM roadmap: swap 5 near-synonym keywords for distinct topics
Replace cannibalization-risk near-duplicates (cloud based pacs system,
healthcare data integration, medical image management, dicom reader software,
dicom viewer program) with distinct topics (DICOM standard, routing, toolkit/SDK,
PACS integration, FHIR). Still 90 articles, 30/30/30. All keywords/titles unique.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/ebm/keyword-research.xlsx
+++ b/decks/ebm/keyword-research.xlsx
@@ -1740,28 +1740,28 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Cloud-Based PACS: Architecture and Benefits</t>
+          <t>The DICOM Standard: A Practical Overview</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>cloud based pacs system</t>
+          <t>dicom standard</t>
         </is>
       </c>
       <c r="D27" s="4" t="n">
         <v>140</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G27" s="11" t="inlineStr">
-        <is>
-          <t>Cloud, AI &amp; Compliance</t>
+        <v>32</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>Standards &amp; Interoperability</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1828,28 +1828,28 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Medical Image Management, Explained</t>
+          <t>DICOMweb Explained: WADO, STOW, and QIDO</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>medical image management</t>
+          <t>dicomweb</t>
         </is>
       </c>
       <c r="D29" s="4" t="n">
         <v>90</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>DICOM Viewers &amp; Image Access</t>
+        <v>41</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>Standards &amp; Interoperability</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1872,28 +1872,28 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DICOMweb Explained: WADO, STOW, and QIDO</t>
+          <t>Reading DICOM on iPad: From Free Apps to FDA Class II</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>dicomweb</t>
+          <t>free dicom viewer ipad</t>
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G30" s="12" t="inlineStr">
-        <is>
-          <t>Standards &amp; Interoperability</t>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>DICOM Viewers &amp; Image Access</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1916,23 +1916,23 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Reading DICOM on iPad: From Free Apps to FDA Class II</t>
+          <t>DICOM Toolkits &amp; SDKs: Embedding Imaging Into Your Product</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>free dicom viewer ipad</t>
+          <t>dicom toolkit</t>
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="F31" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>18</v>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -1942,12 +1942,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="J31" s="2" t="n">
@@ -2400,28 +2400,28 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Healthcare Data Integration for Imaging Platforms</t>
+          <t>How Secure Medical Image Sharing Works</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>healthcare data integration</t>
+          <t>medical image sharing</t>
         </is>
       </c>
       <c r="D42" s="4" t="n">
-        <v>390</v>
+        <v>320</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G42" s="12" t="inlineStr">
-        <is>
-          <t>Standards &amp; Interoperability</t>
+        <v>31</v>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>DICOM Viewers &amp; Image Access</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2444,38 +2444,38 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>How Secure Medical Image Sharing Works</t>
+          <t>Build Imaging Software Without Building a PACS From Scratch</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>medical image sharing</t>
+          <t>medical imaging software development</t>
         </is>
       </c>
       <c r="D43" s="4" t="n">
         <v>320</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="F43" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>DICOM Viewers &amp; Image Access</t>
+        <v>7</v>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>PACS Platform &amp; Deployment</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="J43" s="2" t="n">
@@ -2488,38 +2488,38 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Build Imaging Software Without Building a PACS From Scratch</t>
+          <t>AI in Pathology and Imaging: The Overlap</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>medical imaging software development</t>
+          <t>ai in pathology</t>
         </is>
       </c>
       <c r="D44" s="4" t="n">
-        <v>320</v>
+        <v>260</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="F44" s="10" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="G44" s="8" t="inlineStr">
-        <is>
-          <t>PACS Platform &amp; Deployment</t>
+        <v>51</v>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>Cloud, AI &amp; Compliance</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J44" s="2" t="n">
@@ -2532,28 +2532,28 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>AI in Pathology and Imaging: The Overlap</t>
+          <t>PACS at the Point of Diagnosis: What Radiologists Need</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>ai in pathology</t>
+          <t>pacs diagnostic imaging</t>
         </is>
       </c>
       <c r="D45" s="4" t="n">
         <v>260</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="G45" s="11" t="inlineStr">
-        <is>
-          <t>Cloud, AI &amp; Compliance</t>
+        <v>28</v>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>PACS Platform &amp; Deployment</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2576,28 +2576,28 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PACS at the Point of Diagnosis: What Radiologists Need</t>
+          <t>How Integration Engines Route Clinical Data</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>pacs diagnostic imaging</t>
+          <t>healthcare integration engine</t>
         </is>
       </c>
       <c r="D46" s="4" t="n">
-        <v>260</v>
+        <v>210</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G46" s="8" t="inlineStr">
-        <is>
-          <t>PACS Platform &amp; Deployment</t>
+        <v>17</v>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>Standards &amp; Interoperability</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2620,28 +2620,28 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>How Integration Engines Route Clinical Data</t>
+          <t>Cloud Viewers: Streaming Studies on Any Device</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>healthcare integration engine</t>
+          <t>cloud viewer</t>
         </is>
       </c>
       <c r="D47" s="4" t="n">
-        <v>210</v>
+        <v>170</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
       </c>
-      <c r="G47" s="12" t="inlineStr">
-        <is>
-          <t>Standards &amp; Interoperability</t>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>DICOM Viewers &amp; Image Access</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2664,28 +2664,28 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cloud Viewers: Streaming Studies on Any Device</t>
+          <t>HL7 Integration Engines: Mirth and the Alternatives</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>cloud viewer</t>
+          <t>hl7 integration engine</t>
         </is>
       </c>
       <c r="D48" s="4" t="n">
         <v>170</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F48" s="10" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
       </c>
-      <c r="G48" s="6" t="inlineStr">
-        <is>
-          <t>DICOM Viewers &amp; Image Access</t>
+      <c r="G48" s="12" t="inlineStr">
+        <is>
+          <t>Standards &amp; Interoperability</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2708,23 +2708,23 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>HL7 Integration Engines: Mirth and the Alternatives</t>
+          <t>The Payoff of EHR Interoperability</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>hl7 integration engine</t>
+          <t>benefits of ehr interoperability</t>
         </is>
       </c>
       <c r="D49" s="4" t="n">
         <v>170</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="F49" s="10" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>29</v>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G49" s="12" t="inlineStr">
@@ -2734,12 +2734,12 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J49" s="2" t="n">
@@ -2752,38 +2752,38 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>The Payoff of EHR Interoperability</t>
+          <t>Freeware DICOM Viewers vs Diagnostic-Grade: The Real Differences</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>benefits of ehr interoperability</t>
+          <t>dicom viewer freeware</t>
         </is>
       </c>
       <c r="D50" s="4" t="n">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="F50" s="7" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G50" s="12" t="inlineStr">
-        <is>
-          <t>Standards &amp; Interoperability</t>
+        <v>40</v>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>DICOM Viewers &amp; Image Access</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J50" s="2" t="n">
@@ -2796,19 +2796,19 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Freeware DICOM Viewers vs Diagnostic-Grade: The Real Differences</t>
+          <t>Web DICOM Viewers: Zero-Footprint Image Access</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>dicom viewer freeware</t>
+          <t>dicom web viewer</t>
         </is>
       </c>
       <c r="D51" s="4" t="n">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
@@ -2840,28 +2840,28 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Web DICOM Viewers: Zero-Footprint Image Access</t>
+          <t>PACS Integration: Connecting Modalities, RIS, and EHR</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>dicom web viewer</t>
+          <t>pacs integration</t>
         </is>
       </c>
       <c r="D52" s="4" t="n">
         <v>110</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="F52" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>DICOM Viewers &amp; Image Access</t>
+        <v>13</v>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>Standards &amp; Interoperability</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3896,19 +3896,19 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>VNA in Imaging: Consolidating Studies Across Systems</t>
+          <t>DICOM Routing: Moving Studies Between Systems</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>vna imaging</t>
+          <t>dicom router</t>
         </is>
       </c>
       <c r="D76" s="4" t="n">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
@@ -3940,38 +3940,38 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Choosing an Image-Sharing Platform for Teleradiology</t>
+          <t>FHIR for Imaging: How FHIR Resources Model Medical Data</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>best dicom image sharing platform for teleradiology providers</t>
+          <t>fhir resource</t>
         </is>
       </c>
       <c r="D77" s="4" t="n">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="F77" s="7" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G77" s="6" t="inlineStr">
-        <is>
-          <t>DICOM Viewers &amp; Image Access</t>
+        <v>33</v>
+      </c>
+      <c r="F77" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="G77" s="12" t="inlineStr">
+        <is>
+          <t>Standards &amp; Interoperability</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J77" s="2" t="n">
@@ -3984,16 +3984,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Cloud PACS Vendors: An OEM's Evaluation Framework</t>
+          <t>VNA in Imaging: Consolidating Studies Across Systems</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>cloud pacs vendors</t>
+          <t>vna imaging</t>
         </is>
       </c>
       <c r="D78" s="4" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>15</v>
@@ -4003,19 +4003,19 @@
           <t>Very Easy</t>
         </is>
       </c>
-      <c r="G78" s="11" t="inlineStr">
-        <is>
-          <t>Cloud, AI &amp; Compliance</t>
+      <c r="G78" s="12" t="inlineStr">
+        <is>
+          <t>Standards &amp; Interoperability</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J78" s="2" t="n">
@@ -4028,28 +4028,28 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Evaluating VNA Vendors for a Partner Platform</t>
+          <t>Choosing an Image-Sharing Platform for Teleradiology</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>vna vendors</t>
+          <t>best dicom image sharing platform for teleradiology providers</t>
         </is>
       </c>
       <c r="D79" s="4" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="F79" s="10" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="G79" s="11" t="inlineStr">
-        <is>
-          <t>Cloud, AI &amp; Compliance</t>
+        <v>21</v>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>DICOM Viewers &amp; Image Access</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -4072,23 +4072,23 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>AI Radiology Solutions: Matching Tools to Workflows</t>
+          <t>Cloud PACS Vendors: An OEM's Evaluation Framework</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>ai radiology solutions</t>
+          <t>cloud pacs vendors</t>
         </is>
       </c>
       <c r="D80" s="4" t="n">
         <v>50</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="F80" s="5" t="inlineStr">
-        <is>
-          <t>Hard</t>
+        <v>15</v>
+      </c>
+      <c r="F80" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G80" s="11" t="inlineStr">
@@ -4098,12 +4098,12 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="J80" s="2" t="n">
@@ -4116,38 +4116,38 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>How to Share Medical Images Securely and Compliantly</t>
+          <t>Evaluating VNA Vendors for a Partner Platform</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>share medical images</t>
+          <t>vna vendors</t>
         </is>
       </c>
       <c r="D81" s="4" t="n">
         <v>50</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="F81" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="G81" s="6" t="inlineStr">
-        <is>
-          <t>DICOM Viewers &amp; Image Access</t>
+        <v>13</v>
+      </c>
+      <c r="F81" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G81" s="11" t="inlineStr">
+        <is>
+          <t>Cloud, AI &amp; Compliance</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="J81" s="2" t="n">
@@ -4160,28 +4160,28 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Radiology Image Sharing Platforms: A Practical Overview</t>
+          <t>AI Radiology Solutions: Matching Tools to Workflows</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>radiology image sharing platforms</t>
+          <t>ai radiology solutions</t>
         </is>
       </c>
       <c r="D82" s="4" t="n">
         <v>50</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="F82" s="10" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="G82" s="6" t="inlineStr">
-        <is>
-          <t>DICOM Viewers &amp; Image Access</t>
+        <v>62</v>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G82" s="11" t="inlineStr">
+        <is>
+          <t>Cloud, AI &amp; Compliance</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -4204,23 +4204,23 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Diagnostic Image Viewers: The Workstation in the Browser</t>
+          <t>How to Share Medical Images Securely and Compliantly</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>medical image viewer</t>
+          <t>share medical images</t>
         </is>
       </c>
       <c r="D83" s="4" t="n">
         <v>50</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>56</v>
-      </c>
-      <c r="F83" s="5" t="inlineStr">
-        <is>
-          <t>Hard</t>
+        <v>40</v>
+      </c>
+      <c r="F83" s="9" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G83" s="6" t="inlineStr">
@@ -4248,38 +4248,38 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PACS vs VNA: Storage Strategies Compared</t>
+          <t>Radiology Image Sharing Platforms: A Practical Overview</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>pacs vs vna</t>
+          <t>radiology image sharing platforms</t>
         </is>
       </c>
       <c r="D84" s="4" t="n">
         <v>50</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
       </c>
-      <c r="G84" s="12" t="inlineStr">
-        <is>
-          <t>Standards &amp; Interoperability</t>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>DICOM Viewers &amp; Image Access</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J84" s="2" t="n">
@@ -4292,23 +4292,23 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>DICOM Viewers on Android: What's Possible</t>
+          <t>Diagnostic Image Viewers: The Workstation in the Browser</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>dicom viewer android</t>
+          <t>medical image viewer</t>
         </is>
       </c>
       <c r="D85" s="4" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="F85" s="10" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>56</v>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr">
@@ -4336,28 +4336,28 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>DICOM Reader Software Compared</t>
+          <t>PACS vs VNA: Storage Strategies Compared</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>dicom reader software</t>
+          <t>pacs vs vna</t>
         </is>
       </c>
       <c r="D86" s="4" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="F86" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="G86" s="6" t="inlineStr">
-        <is>
-          <t>DICOM Viewers &amp; Image Access</t>
+        <v>2</v>
+      </c>
+      <c r="F86" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G86" s="12" t="inlineStr">
+        <is>
+          <t>Standards &amp; Interoperability</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4380,23 +4380,23 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Picking a DICOM Viewer for Your Own Product</t>
+          <t>DICOM Viewers on Android: What's Possible</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>dicom viewer program</t>
+          <t>dicom viewer android</t>
         </is>
       </c>
       <c r="D87" s="4" t="n">
         <v>40</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="F87" s="9" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>8</v>
+      </c>
+      <c r="F87" s="10" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G87" s="6" t="inlineStr">
@@ -4406,12 +4406,12 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J87" s="2" t="n">
@@ -6496,9 +6496,9 @@
           <t>Middle of funnel</t>
         </is>
       </c>
-      <c r="G57" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G57" s="13" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -9532,9 +9532,9 @@
           <t>Middle of funnel</t>
         </is>
       </c>
-      <c r="G149" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G149" s="13" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -10489,9 +10489,9 @@
           <t>Middle of funnel</t>
         </is>
       </c>
-      <c r="G178" s="13" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G178" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -10654,9 +10654,9 @@
           <t>Middle of funnel</t>
         </is>
       </c>
-      <c r="G183" s="13" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G183" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -12106,9 +12106,9 @@
           <t>Middle of funnel</t>
         </is>
       </c>
-      <c r="G227" s="13" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G227" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -12139,9 +12139,9 @@
           <t>Top of funnel</t>
         </is>
       </c>
-      <c r="G228" s="13" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G228" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -13987,9 +13987,9 @@
           <t>Middle of funnel</t>
         </is>
       </c>
-      <c r="G284" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G284" s="13" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -24250,9 +24250,9 @@
           <t>Middle of funnel</t>
         </is>
       </c>
-      <c r="G595" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G595" s="13" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -24349,9 +24349,9 @@
           <t>Bottom of funnel</t>
         </is>
       </c>
-      <c r="G598" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G598" s="13" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -27385,9 +27385,9 @@
           <t>Top of funnel</t>
         </is>
       </c>
-      <c r="G690" s="13" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G690" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -29134,9 +29134,9 @@
       <c r="A23" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  90 articles, split exactly 30/30/30 across Months 1–3
-  38,360 total monthly searches addressed
+  38,190 total monthly searches addressed
   42 easy wins at KD &lt;= 25 — front-loaded so a brand-new domain sees rankings early
-  Average difficulty KD 29 — deliberately achievable for a launching site</t>
+  Average difficulty KD 28 — deliberately achievable for a launching site</t>
         </is>
       </c>
     </row>

</xml_diff>